<commit_message>
removed empty column sgpi
</commit_message>
<xml_diff>
--- a/FORMAT.xlsx
+++ b/FORMAT.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\himan\OneDrive\Desktop\Projects\Smart-Data-Management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RAJ\Desktop\Intern\Smart-Data-Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9798CD86-3AE0-49E0-A8A3-9F070CE1EE90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{994EE4FC-5708-4B1D-8E29-78FA3F483F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F48298C6-7D83-413E-BD9E-10C084A6DE08}"/>
   </bookViews>
@@ -27,7 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="155">
   <si>
     <t>SEMESTER</t>
   </si>
@@ -290,9 +289,6 @@
   </si>
   <si>
     <t>SECURED_MARKS</t>
-  </si>
-  <si>
-    <t>SGPI</t>
   </si>
   <si>
     <t>Environmental studies</t>
@@ -872,7 +868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91149176-0434-4170-AB38-CDBFCEE8D501}">
-  <dimension ref="A1:AU26"/>
+  <dimension ref="A1:AT26"/>
   <sheetFormatPr defaultColWidth="23.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -920,16 +916,15 @@
     <col min="43" max="43" width="14" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="5" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="7.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>5</v>
@@ -941,16 +936,16 @@
         <v>7</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>126</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>127</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>47</v>
@@ -1037,7 +1032,7 @@
         <v>72</v>
       </c>
       <c r="AL1" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AM1" s="4" t="s">
         <v>79</v>
@@ -1061,13 +1056,10 @@
         <v>2</v>
       </c>
       <c r="AT1" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="AU1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1081,10 +1073,10 @@
         <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G2" s="3">
         <v>38838</v>
@@ -1094,13 +1086,13 @@
         <v>ABC-112233</v>
       </c>
       <c r="I2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J2" s="1">
         <v>43952</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L2">
         <v>1</v>
@@ -1181,7 +1173,7 @@
         <v>15</v>
       </c>
       <c r="AL2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM2">
         <v>35</v>
@@ -1206,11 +1198,11 @@
         <f>AR2/AQ2*100</f>
         <v>82.399999999999991</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AT2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1227,7 +1219,7 @@
         <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G3" s="3">
         <v>38839</v>
@@ -1237,13 +1229,13 @@
         <v>ABC-112234</v>
       </c>
       <c r="I3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J3" s="1">
         <v>43952</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L3">
         <v>1</v>
@@ -1324,7 +1316,7 @@
         <v>10</v>
       </c>
       <c r="AL3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM3">
         <v>58</v>
@@ -1349,11 +1341,11 @@
         <f t="shared" ref="AS3:AS14" si="2">AR3/AQ3*100</f>
         <v>75.599999999999994</v>
       </c>
-      <c r="AU3" t="s">
+      <c r="AT3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1370,7 +1362,7 @@
         <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G4" s="3">
         <v>38840</v>
@@ -1380,13 +1372,13 @@
         <v>ABC-112235</v>
       </c>
       <c r="I4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J4" s="1">
         <v>43952</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L4">
         <v>1</v>
@@ -1467,7 +1459,7 @@
         <v>22</v>
       </c>
       <c r="AL4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM4">
         <v>73</v>
@@ -1492,11 +1484,11 @@
         <f t="shared" si="2"/>
         <v>85.333333333333343</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AT4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1513,7 +1505,7 @@
         <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G5" s="3">
         <v>38841</v>
@@ -1523,13 +1515,13 @@
         <v>ABC-112236</v>
       </c>
       <c r="I5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J5" s="1">
         <v>43952</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L5">
         <v>1</v>
@@ -1610,7 +1602,7 @@
         <v>15</v>
       </c>
       <c r="AL5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM5">
         <v>32</v>
@@ -1635,11 +1627,11 @@
         <f t="shared" si="2"/>
         <v>80.666666666666657</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AT5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1656,7 +1648,7 @@
         <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G6" s="3">
         <v>38842</v>
@@ -1666,13 +1658,13 @@
         <v>ABC-112237</v>
       </c>
       <c r="I6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J6" s="1">
         <v>43952</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L6">
         <v>1</v>
@@ -1753,7 +1745,7 @@
         <v>10</v>
       </c>
       <c r="AL6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM6">
         <v>35</v>
@@ -1778,11 +1770,11 @@
         <f t="shared" si="2"/>
         <v>68.400000000000006</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AT6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1799,7 +1791,7 @@
         <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G7" s="3">
         <v>38843</v>
@@ -1809,13 +1801,13 @@
         <v>ABC-112238</v>
       </c>
       <c r="I7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J7" s="1">
         <v>43952</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L7">
         <v>1</v>
@@ -1896,7 +1888,7 @@
         <v>23</v>
       </c>
       <c r="AL7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM7">
         <v>58</v>
@@ -1921,11 +1913,11 @@
         <f t="shared" si="2"/>
         <v>88.533333333333331</v>
       </c>
-      <c r="AU7" t="s">
+      <c r="AT7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1942,7 +1934,7 @@
         <v>32</v>
       </c>
       <c r="F8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G8" s="3">
         <v>38844</v>
@@ -1952,13 +1944,13 @@
         <v>ABC-112239</v>
       </c>
       <c r="I8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J8" s="1">
         <v>43952</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L8">
         <v>1</v>
@@ -2039,7 +2031,7 @@
         <v>22</v>
       </c>
       <c r="AL8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM8">
         <v>73</v>
@@ -2064,11 +2056,11 @@
         <f t="shared" si="2"/>
         <v>82.13333333333334</v>
       </c>
-      <c r="AU8" t="s">
+      <c r="AT8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2085,7 +2077,7 @@
         <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G9" s="3">
         <v>38845</v>
@@ -2095,13 +2087,13 @@
         <v>ABC-112240</v>
       </c>
       <c r="I9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J9" s="1">
         <v>43952</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L9">
         <v>1</v>
@@ -2182,7 +2174,7 @@
         <v>20</v>
       </c>
       <c r="AL9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM9">
         <v>32</v>
@@ -2207,11 +2199,11 @@
         <f t="shared" si="2"/>
         <v>72.266666666666666</v>
       </c>
-      <c r="AU9" t="s">
+      <c r="AT9" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2228,7 +2220,7 @@
         <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G10" s="3">
         <v>38846</v>
@@ -2238,13 +2230,13 @@
         <v>ABC-112241</v>
       </c>
       <c r="I10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J10" s="1">
         <v>43952</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L10">
         <v>1</v>
@@ -2325,7 +2317,7 @@
         <v>15</v>
       </c>
       <c r="AL10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM10">
         <v>35</v>
@@ -2350,11 +2342,11 @@
         <f t="shared" si="2"/>
         <v>79.2</v>
       </c>
-      <c r="AU10" t="s">
+      <c r="AT10" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2371,7 +2363,7 @@
         <v>38</v>
       </c>
       <c r="F11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G11" s="3">
         <v>38847</v>
@@ -2381,13 +2373,13 @@
         <v>ABC-112242</v>
       </c>
       <c r="I11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J11" s="1">
         <v>43952</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L11">
         <v>1</v>
@@ -2468,7 +2460,7 @@
         <v>10</v>
       </c>
       <c r="AL11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM11">
         <v>58</v>
@@ -2493,11 +2485,11 @@
         <f t="shared" si="2"/>
         <v>86.133333333333326</v>
       </c>
-      <c r="AU11" t="s">
+      <c r="AT11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2514,7 +2506,7 @@
         <v>40</v>
       </c>
       <c r="F12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G12" s="3">
         <v>38848</v>
@@ -2524,13 +2516,13 @@
         <v>ABC-112243</v>
       </c>
       <c r="I12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J12" s="1">
         <v>43952</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L12">
         <v>1</v>
@@ -2611,7 +2603,7 @@
         <v>10</v>
       </c>
       <c r="AL12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM12">
         <v>73</v>
@@ -2636,11 +2628,11 @@
         <f t="shared" si="2"/>
         <v>88.4</v>
       </c>
-      <c r="AU12" t="s">
+      <c r="AT12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2657,7 +2649,7 @@
         <v>42</v>
       </c>
       <c r="F13" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G13" s="3">
         <v>38849</v>
@@ -2667,13 +2659,13 @@
         <v>ABC-112244</v>
       </c>
       <c r="I13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J13" s="1">
         <v>43952</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L13">
         <v>1</v>
@@ -2754,7 +2746,7 @@
         <v>23</v>
       </c>
       <c r="AL13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM13">
         <v>32</v>
@@ -2779,11 +2771,11 @@
         <f t="shared" si="2"/>
         <v>78.400000000000006</v>
       </c>
-      <c r="AU13" t="s">
+      <c r="AT13" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2800,7 +2792,7 @@
         <v>44</v>
       </c>
       <c r="F14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G14" s="3">
         <v>38850</v>
@@ -2810,13 +2802,13 @@
         <v>ABC-112245</v>
       </c>
       <c r="I14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J14" s="1">
         <v>43952</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L14">
         <v>1</v>
@@ -2897,7 +2889,7 @@
         <v>22</v>
       </c>
       <c r="AL14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM14">
         <v>35</v>
@@ -2922,11 +2914,11 @@
         <f t="shared" si="2"/>
         <v>72.8</v>
       </c>
-      <c r="AU14" t="s">
+      <c r="AT14" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2934,16 +2926,16 @@
         <v>112246</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E15" t="s">
         <v>46</v>
       </c>
       <c r="F15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G15" s="3">
         <v>38851</v>
@@ -2953,13 +2945,13 @@
         <v>ABC-112246</v>
       </c>
       <c r="I15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J15" s="1">
         <v>43952</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L15">
         <v>1</v>
@@ -3040,7 +3032,7 @@
         <v>15</v>
       </c>
       <c r="AL15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM15">
         <v>35</v>
@@ -3065,11 +3057,11 @@
         <f>AR15/AQ15*100</f>
         <v>82.399999999999991</v>
       </c>
-      <c r="AU15" t="s">
+      <c r="AT15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3077,16 +3069,16 @@
         <v>112247</v>
       </c>
       <c r="C16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G16" s="3">
         <v>38852</v>
@@ -3096,13 +3088,13 @@
         <v>ABC-112247</v>
       </c>
       <c r="I16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J16" s="1">
         <v>43952</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L16">
         <v>1</v>
@@ -3183,7 +3175,7 @@
         <v>10</v>
       </c>
       <c r="AL16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM16">
         <v>58</v>
@@ -3208,11 +3200,11 @@
         <f t="shared" ref="AS16:AS26" si="4">AR16/AQ16*100</f>
         <v>75.599999999999994</v>
       </c>
-      <c r="AU16" t="s">
+      <c r="AT16" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3220,16 +3212,16 @@
         <v>112248</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G17" s="3">
         <v>38853</v>
@@ -3239,13 +3231,13 @@
         <v>ABC-112248</v>
       </c>
       <c r="I17" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J17" s="1">
         <v>43952</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L17">
         <v>1</v>
@@ -3326,7 +3318,7 @@
         <v>22</v>
       </c>
       <c r="AL17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM17">
         <v>73</v>
@@ -3351,11 +3343,11 @@
         <f t="shared" si="4"/>
         <v>85.333333333333343</v>
       </c>
-      <c r="AU17" t="s">
+      <c r="AT17" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3363,16 +3355,16 @@
         <v>112249</v>
       </c>
       <c r="C18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G18" s="3">
         <v>38854</v>
@@ -3382,13 +3374,13 @@
         <v>ABC-112249</v>
       </c>
       <c r="I18" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J18" s="1">
         <v>43952</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L18">
         <v>1</v>
@@ -3469,7 +3461,7 @@
         <v>15</v>
       </c>
       <c r="AL18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM18">
         <v>32</v>
@@ -3494,11 +3486,11 @@
         <f t="shared" si="4"/>
         <v>80.666666666666657</v>
       </c>
-      <c r="AU18" t="s">
+      <c r="AT18" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3506,16 +3498,16 @@
         <v>112250</v>
       </c>
       <c r="C19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F19" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G19" s="3">
         <v>38855</v>
@@ -3525,13 +3517,13 @@
         <v>ABC-112250</v>
       </c>
       <c r="I19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J19" s="1">
         <v>43952</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L19">
         <v>1</v>
@@ -3612,7 +3604,7 @@
         <v>10</v>
       </c>
       <c r="AL19" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM19">
         <v>35</v>
@@ -3637,11 +3629,11 @@
         <f t="shared" si="4"/>
         <v>68.400000000000006</v>
       </c>
-      <c r="AU19" t="s">
+      <c r="AT19" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3649,16 +3641,16 @@
         <v>112251</v>
       </c>
       <c r="C20" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D20" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F20" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G20" s="3">
         <v>38856</v>
@@ -3668,13 +3660,13 @@
         <v>ABC-112251</v>
       </c>
       <c r="I20" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J20" s="1">
         <v>43952</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L20">
         <v>1</v>
@@ -3755,7 +3747,7 @@
         <v>23</v>
       </c>
       <c r="AL20" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM20">
         <v>58</v>
@@ -3780,11 +3772,11 @@
         <f t="shared" si="4"/>
         <v>88.533333333333331</v>
       </c>
-      <c r="AU20" t="s">
+      <c r="AT20" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3792,16 +3784,16 @@
         <v>112252</v>
       </c>
       <c r="C21" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E21" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F21" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G21" s="3">
         <v>38857</v>
@@ -3811,13 +3803,13 @@
         <v>ABC-112252</v>
       </c>
       <c r="I21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J21" s="1">
         <v>43952</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L21">
         <v>1</v>
@@ -3898,7 +3890,7 @@
         <v>22</v>
       </c>
       <c r="AL21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM21">
         <v>73</v>
@@ -3923,11 +3915,11 @@
         <f t="shared" si="4"/>
         <v>82.13333333333334</v>
       </c>
-      <c r="AU21" t="s">
+      <c r="AT21" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3935,16 +3927,16 @@
         <v>112253</v>
       </c>
       <c r="C22" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D22" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F22" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G22" s="3">
         <v>38858</v>
@@ -3954,13 +3946,13 @@
         <v>ABC-112253</v>
       </c>
       <c r="I22" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J22" s="1">
         <v>43952</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L22">
         <v>1</v>
@@ -4041,7 +4033,7 @@
         <v>20</v>
       </c>
       <c r="AL22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM22">
         <v>32</v>
@@ -4066,11 +4058,11 @@
         <f t="shared" si="4"/>
         <v>72.266666666666666</v>
       </c>
-      <c r="AU22" t="s">
+      <c r="AT22" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -4078,16 +4070,16 @@
         <v>112254</v>
       </c>
       <c r="C23" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F23" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G23" s="3">
         <v>38859</v>
@@ -4097,13 +4089,13 @@
         <v>ABC-112254</v>
       </c>
       <c r="I23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J23" s="1">
         <v>43952</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L23">
         <v>1</v>
@@ -4184,7 +4176,7 @@
         <v>15</v>
       </c>
       <c r="AL23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM23">
         <v>35</v>
@@ -4209,11 +4201,11 @@
         <f t="shared" si="4"/>
         <v>79.2</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AT23" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -4221,16 +4213,16 @@
         <v>112255</v>
       </c>
       <c r="C24" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D24" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E24" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G24" s="3">
         <v>38860</v>
@@ -4240,13 +4232,13 @@
         <v>ABC-112255</v>
       </c>
       <c r="I24" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J24" s="1">
         <v>43952</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L24">
         <v>1</v>
@@ -4327,7 +4319,7 @@
         <v>10</v>
       </c>
       <c r="AL24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM24">
         <v>58</v>
@@ -4352,11 +4344,11 @@
         <f t="shared" si="4"/>
         <v>86.133333333333326</v>
       </c>
-      <c r="AU24" t="s">
+      <c r="AT24" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -4364,16 +4356,16 @@
         <v>112256</v>
       </c>
       <c r="C25" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D25" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E25" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F25" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G25" s="3">
         <v>38861</v>
@@ -4383,13 +4375,13 @@
         <v>ABC-112256</v>
       </c>
       <c r="I25" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J25" s="1">
         <v>43952</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L25">
         <v>1</v>
@@ -4470,7 +4462,7 @@
         <v>10</v>
       </c>
       <c r="AL25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM25">
         <v>73</v>
@@ -4495,11 +4487,11 @@
         <f t="shared" si="4"/>
         <v>88.4</v>
       </c>
-      <c r="AU25" t="s">
+      <c r="AT25" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:46" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -4507,16 +4499,16 @@
         <v>112257</v>
       </c>
       <c r="C26" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G26" s="3">
         <v>38862</v>
@@ -4526,13 +4518,13 @@
         <v>ABC-112257</v>
       </c>
       <c r="I26" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J26" s="1">
         <v>43952</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L26">
         <v>1</v>
@@ -4613,7 +4605,7 @@
         <v>23</v>
       </c>
       <c r="AL26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AM26">
         <v>32</v>
@@ -4638,7 +4630,7 @@
         <f t="shared" si="4"/>
         <v>78.400000000000006</v>
       </c>
-      <c r="AU26" t="s">
+      <c r="AT26" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
change -ORAL to _ORAL
</commit_message>
<xml_diff>
--- a/FORMAT.xlsx
+++ b/FORMAT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RAJ\Desktop\Intern\Smart-Data-Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{994EE4FC-5708-4B1D-8E29-78FA3F483F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BDB4707-8015-4036-A65D-BDBEFE7F2822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F48298C6-7D83-413E-BD9E-10C084A6DE08}"/>
   </bookViews>
@@ -189,9 +189,6 @@
     <t>SUB_1_INTERNAL</t>
   </si>
   <si>
-    <t>SUB_1_PRACTICAL-ORAL</t>
-  </si>
-  <si>
     <t>SUB_1_NAME</t>
   </si>
   <si>
@@ -204,9 +201,6 @@
     <t>SUB_2_INTERNAL</t>
   </si>
   <si>
-    <t>SUB_2_PRACTICAL-ORAL</t>
-  </si>
-  <si>
     <t>SUB_2_TERM_WORK</t>
   </si>
   <si>
@@ -216,9 +210,6 @@
     <t>SUB_3_INTERNAL</t>
   </si>
   <si>
-    <t>SUB_3_PRACTICAL-ORAL</t>
-  </si>
-  <si>
     <t>SUB_3_TERM_WORK</t>
   </si>
   <si>
@@ -234,9 +225,6 @@
     <t>SUB_4_INTERNAL</t>
   </si>
   <si>
-    <t>SUB_4_PRACTICAL-ORAL</t>
-  </si>
-  <si>
     <t>SUB_4_TERM_WORK</t>
   </si>
   <si>
@@ -249,9 +237,6 @@
     <t>SUB_5_INTERNAL</t>
   </si>
   <si>
-    <t>SUB_5_PRACTICAL-ORAL</t>
-  </si>
-  <si>
     <t>SUB_5_TERM_WORK</t>
   </si>
   <si>
@@ -279,9 +264,6 @@
     <t>SUB_6_INTERNAL</t>
   </si>
   <si>
-    <t>SUB_6_PRACTICAL-ORAL</t>
-  </si>
-  <si>
     <t>SUB_6_TERM_WORK</t>
   </si>
   <si>
@@ -499,6 +481,24 @@
   </si>
   <si>
     <t>LAST_NAME1</t>
+  </si>
+  <si>
+    <t>SUB_1_PRACTICAL_ORAL</t>
+  </si>
+  <si>
+    <t>SUB_2_PRACTICAL_ORAL</t>
+  </si>
+  <si>
+    <t>SUB_3_PRACTICAL_ORAL</t>
+  </si>
+  <si>
+    <t>SUB_4_PRACTICAL_ORAL</t>
+  </si>
+  <si>
+    <t>SUB_5_PRACTICAL_ORAL</t>
+  </si>
+  <si>
+    <t>SUB_6_PRACTICAL_ORAL</t>
   </si>
 </sst>
 </file>
@@ -924,7 +924,7 @@
         <v>4</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>5</v>
@@ -936,28 +936,28 @@
         <v>7</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>47</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="L1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>48</v>
@@ -966,91 +966,91 @@
         <v>50</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>51</v>
+        <v>149</v>
       </c>
       <c r="Q1" s="4" t="s">
         <v>49</v>
       </c>
       <c r="R1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="S1" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="T1" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="U1" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="V1" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="W1" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="X1" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="Y1" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="Z1" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="AA1" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB1" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC1" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="AD1" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="X1" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB1" s="4" t="s">
+      <c r="AE1" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="AF1" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="AC1" s="4" t="s">
+      <c r="AG1" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="AD1" s="4" t="s">
+      <c r="AH1" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="AE1" s="4" t="s">
+      <c r="AI1" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="AF1" s="4" t="s">
+      <c r="AJ1" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="AK1" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AG1" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="AH1" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="AI1" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="AJ1" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="AK1" s="4" t="s">
-        <v>72</v>
-      </c>
       <c r="AL1" s="4" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="AM1" s="4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="AN1" s="4" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="AO1" s="4" t="s">
-        <v>81</v>
+        <v>154</v>
       </c>
       <c r="AP1" s="4" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AQ1" s="4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AR1" s="4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AS1" s="4" t="s">
         <v>2</v>
@@ -1073,10 +1073,10 @@
         <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="F2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G2" s="3">
         <v>38838</v>
@@ -1086,19 +1086,19 @@
         <v>ABC-112233</v>
       </c>
       <c r="I2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J2" s="1">
         <v>43952</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N2">
         <v>45</v>
@@ -1113,7 +1113,7 @@
         <v>17</v>
       </c>
       <c r="R2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S2">
         <v>68</v>
@@ -1128,7 +1128,7 @@
         <v>24</v>
       </c>
       <c r="W2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X2">
         <v>73</v>
@@ -1143,7 +1143,7 @@
         <v>23</v>
       </c>
       <c r="AB2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC2">
         <v>35</v>
@@ -1158,7 +1158,7 @@
         <v>20</v>
       </c>
       <c r="AG2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH2">
         <v>52</v>
@@ -1173,7 +1173,7 @@
         <v>15</v>
       </c>
       <c r="AL2" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM2">
         <v>35</v>
@@ -1219,7 +1219,7 @@
         <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="G3" s="3">
         <v>38839</v>
@@ -1229,19 +1229,19 @@
         <v>ABC-112234</v>
       </c>
       <c r="I3" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J3" s="1">
         <v>43952</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N3">
         <v>14</v>
@@ -1256,7 +1256,7 @@
         <v>20</v>
       </c>
       <c r="R3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S3">
         <v>39</v>
@@ -1271,7 +1271,7 @@
         <v>18</v>
       </c>
       <c r="W3" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X3">
         <v>58</v>
@@ -1286,7 +1286,7 @@
         <v>10</v>
       </c>
       <c r="AB3" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC3">
         <v>52</v>
@@ -1301,7 +1301,7 @@
         <v>15</v>
       </c>
       <c r="AG3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH3">
         <v>58</v>
@@ -1316,7 +1316,7 @@
         <v>10</v>
       </c>
       <c r="AL3" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM3">
         <v>58</v>
@@ -1362,7 +1362,7 @@
         <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="G4" s="3">
         <v>38840</v>
@@ -1372,19 +1372,19 @@
         <v>ABC-112235</v>
       </c>
       <c r="I4" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J4" s="1">
         <v>43952</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N4">
         <v>32</v>
@@ -1399,7 +1399,7 @@
         <v>23</v>
       </c>
       <c r="R4" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S4">
         <v>52</v>
@@ -1414,7 +1414,7 @@
         <v>15</v>
       </c>
       <c r="W4" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X4">
         <v>42</v>
@@ -1429,7 +1429,7 @@
         <v>22</v>
       </c>
       <c r="AB4" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC4">
         <v>73</v>
@@ -1444,7 +1444,7 @@
         <v>23</v>
       </c>
       <c r="AG4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH4">
         <v>42</v>
@@ -1459,7 +1459,7 @@
         <v>22</v>
       </c>
       <c r="AL4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM4">
         <v>73</v>
@@ -1505,7 +1505,7 @@
         <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="G5" s="3">
         <v>38841</v>
@@ -1515,19 +1515,19 @@
         <v>ABC-112236</v>
       </c>
       <c r="I5" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J5" s="1">
         <v>43952</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N5">
         <v>54</v>
@@ -1542,7 +1542,7 @@
         <v>22</v>
       </c>
       <c r="R5" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S5">
         <v>73</v>
@@ -1557,7 +1557,7 @@
         <v>23</v>
       </c>
       <c r="W5" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X5">
         <v>32</v>
@@ -1572,7 +1572,7 @@
         <v>22</v>
       </c>
       <c r="AB5" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC5">
         <v>32</v>
@@ -1587,7 +1587,7 @@
         <v>22</v>
       </c>
       <c r="AG5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH5">
         <v>52</v>
@@ -1602,7 +1602,7 @@
         <v>15</v>
       </c>
       <c r="AL5" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM5">
         <v>32</v>
@@ -1648,7 +1648,7 @@
         <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="G6" s="3">
         <v>38842</v>
@@ -1658,19 +1658,19 @@
         <v>ABC-112237</v>
       </c>
       <c r="I6" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J6" s="1">
         <v>43952</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N6">
         <v>16</v>
@@ -1685,7 +1685,7 @@
         <v>19</v>
       </c>
       <c r="R6" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S6">
         <v>58</v>
@@ -1700,7 +1700,7 @@
         <v>10</v>
       </c>
       <c r="W6" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X6">
         <v>35</v>
@@ -1715,7 +1715,7 @@
         <v>20</v>
       </c>
       <c r="AB6" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC6">
         <v>35</v>
@@ -1730,7 +1730,7 @@
         <v>20</v>
       </c>
       <c r="AG6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH6">
         <v>58</v>
@@ -1745,7 +1745,7 @@
         <v>10</v>
       </c>
       <c r="AL6" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM6">
         <v>35</v>
@@ -1791,7 +1791,7 @@
         <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="G7" s="3">
         <v>38843</v>
@@ -1801,19 +1801,19 @@
         <v>ABC-112238</v>
       </c>
       <c r="I7" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J7" s="1">
         <v>43952</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N7">
         <v>68</v>
@@ -1828,7 +1828,7 @@
         <v>24</v>
       </c>
       <c r="R7" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S7">
         <v>42</v>
@@ -1843,7 +1843,7 @@
         <v>22</v>
       </c>
       <c r="W7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X7">
         <v>52</v>
@@ -1858,7 +1858,7 @@
         <v>15</v>
       </c>
       <c r="AB7" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC7">
         <v>52</v>
@@ -1873,7 +1873,7 @@
         <v>15</v>
       </c>
       <c r="AG7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH7">
         <v>73</v>
@@ -1888,7 +1888,7 @@
         <v>23</v>
       </c>
       <c r="AL7" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM7">
         <v>58</v>
@@ -1934,7 +1934,7 @@
         <v>32</v>
       </c>
       <c r="F8" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="G8" s="3">
         <v>38844</v>
@@ -1944,19 +1944,19 @@
         <v>ABC-112239</v>
       </c>
       <c r="I8" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J8" s="1">
         <v>43952</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N8">
         <v>39</v>
@@ -1971,7 +1971,7 @@
         <v>18</v>
       </c>
       <c r="R8" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S8">
         <v>32</v>
@@ -1986,7 +1986,7 @@
         <v>22</v>
       </c>
       <c r="W8" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X8">
         <v>73</v>
@@ -2001,7 +2001,7 @@
         <v>23</v>
       </c>
       <c r="AB8" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC8">
         <v>58</v>
@@ -2016,7 +2016,7 @@
         <v>10</v>
       </c>
       <c r="AG8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH8">
         <v>32</v>
@@ -2031,7 +2031,7 @@
         <v>22</v>
       </c>
       <c r="AL8" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM8">
         <v>73</v>
@@ -2077,7 +2077,7 @@
         <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="G9" s="3">
         <v>38845</v>
@@ -2087,19 +2087,19 @@
         <v>ABC-112240</v>
       </c>
       <c r="I9" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J9" s="1">
         <v>43952</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N9">
         <v>52</v>
@@ -2114,7 +2114,7 @@
         <v>15</v>
       </c>
       <c r="R9" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S9">
         <v>35</v>
@@ -2129,7 +2129,7 @@
         <v>20</v>
       </c>
       <c r="W9" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X9">
         <v>32</v>
@@ -2144,7 +2144,7 @@
         <v>22</v>
       </c>
       <c r="AB9" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC9">
         <v>42</v>
@@ -2159,7 +2159,7 @@
         <v>22</v>
       </c>
       <c r="AG9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH9">
         <v>35</v>
@@ -2174,7 +2174,7 @@
         <v>20</v>
       </c>
       <c r="AL9" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM9">
         <v>32</v>
@@ -2220,7 +2220,7 @@
         <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="G10" s="3">
         <v>38846</v>
@@ -2230,19 +2230,19 @@
         <v>ABC-112241</v>
       </c>
       <c r="I10" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J10" s="1">
         <v>43952</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N10">
         <v>73</v>
@@ -2257,7 +2257,7 @@
         <v>23</v>
       </c>
       <c r="R10" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S10">
         <v>52</v>
@@ -2272,7 +2272,7 @@
         <v>15</v>
       </c>
       <c r="W10" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X10">
         <v>35</v>
@@ -2287,7 +2287,7 @@
         <v>20</v>
       </c>
       <c r="AB10" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC10">
         <v>52</v>
@@ -2302,7 +2302,7 @@
         <v>15</v>
       </c>
       <c r="AG10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH10">
         <v>52</v>
@@ -2317,7 +2317,7 @@
         <v>15</v>
       </c>
       <c r="AL10" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM10">
         <v>35</v>
@@ -2363,7 +2363,7 @@
         <v>38</v>
       </c>
       <c r="F11" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="G11" s="3">
         <v>38847</v>
@@ -2373,19 +2373,19 @@
         <v>ABC-112242</v>
       </c>
       <c r="I11" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J11" s="1">
         <v>43952</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N11">
         <v>58</v>
@@ -2400,7 +2400,7 @@
         <v>10</v>
       </c>
       <c r="R11" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S11">
         <v>73</v>
@@ -2415,7 +2415,7 @@
         <v>23</v>
       </c>
       <c r="W11" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X11">
         <v>52</v>
@@ -2430,7 +2430,7 @@
         <v>15</v>
       </c>
       <c r="AB11" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC11">
         <v>58</v>
@@ -2445,7 +2445,7 @@
         <v>10</v>
       </c>
       <c r="AG11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH11">
         <v>58</v>
@@ -2460,7 +2460,7 @@
         <v>10</v>
       </c>
       <c r="AL11" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM11">
         <v>58</v>
@@ -2506,7 +2506,7 @@
         <v>40</v>
       </c>
       <c r="F12" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="G12" s="3">
         <v>38848</v>
@@ -2516,19 +2516,19 @@
         <v>ABC-112243</v>
       </c>
       <c r="I12" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J12" s="1">
         <v>43952</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N12">
         <v>42</v>
@@ -2543,7 +2543,7 @@
         <v>22</v>
       </c>
       <c r="R12" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S12">
         <v>58</v>
@@ -2558,7 +2558,7 @@
         <v>10</v>
       </c>
       <c r="W12" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X12">
         <v>58</v>
@@ -2573,7 +2573,7 @@
         <v>10</v>
       </c>
       <c r="AB12" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC12">
         <v>73</v>
@@ -2588,7 +2588,7 @@
         <v>23</v>
       </c>
       <c r="AG12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH12">
         <v>58</v>
@@ -2603,7 +2603,7 @@
         <v>10</v>
       </c>
       <c r="AL12" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM12">
         <v>73</v>
@@ -2649,7 +2649,7 @@
         <v>42</v>
       </c>
       <c r="F13" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="G13" s="3">
         <v>38849</v>
@@ -2659,19 +2659,19 @@
         <v>ABC-112244</v>
       </c>
       <c r="I13" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J13" s="1">
         <v>43952</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N13">
         <v>32</v>
@@ -2686,7 +2686,7 @@
         <v>22</v>
       </c>
       <c r="R13" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S13">
         <v>42</v>
@@ -2701,7 +2701,7 @@
         <v>22</v>
       </c>
       <c r="W13" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X13">
         <v>42</v>
@@ -2716,7 +2716,7 @@
         <v>22</v>
       </c>
       <c r="AB13" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC13">
         <v>32</v>
@@ -2731,7 +2731,7 @@
         <v>22</v>
       </c>
       <c r="AG13" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH13">
         <v>73</v>
@@ -2746,7 +2746,7 @@
         <v>23</v>
       </c>
       <c r="AL13" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM13">
         <v>32</v>
@@ -2792,7 +2792,7 @@
         <v>44</v>
       </c>
       <c r="F14" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="G14" s="3">
         <v>38850</v>
@@ -2802,19 +2802,19 @@
         <v>ABC-112245</v>
       </c>
       <c r="I14" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J14" s="1">
         <v>43952</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L14">
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N14">
         <v>35</v>
@@ -2829,7 +2829,7 @@
         <v>20</v>
       </c>
       <c r="R14" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S14">
         <v>73</v>
@@ -2844,7 +2844,7 @@
         <v>23</v>
       </c>
       <c r="W14" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X14">
         <v>32</v>
@@ -2859,7 +2859,7 @@
         <v>22</v>
       </c>
       <c r="AB14" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC14">
         <v>35</v>
@@ -2874,7 +2874,7 @@
         <v>20</v>
       </c>
       <c r="AG14" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH14">
         <v>32</v>
@@ -2889,7 +2889,7 @@
         <v>22</v>
       </c>
       <c r="AL14" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM14">
         <v>35</v>
@@ -2926,16 +2926,16 @@
         <v>112246</v>
       </c>
       <c r="C15" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D15" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E15" t="s">
         <v>46</v>
       </c>
       <c r="F15" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="G15" s="3">
         <v>38851</v>
@@ -2945,19 +2945,19 @@
         <v>ABC-112246</v>
       </c>
       <c r="I15" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J15" s="1">
         <v>43952</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L15">
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N15">
         <v>45</v>
@@ -2972,7 +2972,7 @@
         <v>17</v>
       </c>
       <c r="R15" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S15">
         <v>68</v>
@@ -2987,7 +2987,7 @@
         <v>24</v>
       </c>
       <c r="W15" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X15">
         <v>73</v>
@@ -3002,7 +3002,7 @@
         <v>23</v>
       </c>
       <c r="AB15" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC15">
         <v>35</v>
@@ -3017,7 +3017,7 @@
         <v>20</v>
       </c>
       <c r="AG15" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH15">
         <v>52</v>
@@ -3032,7 +3032,7 @@
         <v>15</v>
       </c>
       <c r="AL15" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM15">
         <v>35</v>
@@ -3069,16 +3069,16 @@
         <v>112247</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D16" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E16" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="F16" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="G16" s="3">
         <v>38852</v>
@@ -3088,19 +3088,19 @@
         <v>ABC-112247</v>
       </c>
       <c r="I16" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J16" s="1">
         <v>43952</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L16">
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N16">
         <v>14</v>
@@ -3115,7 +3115,7 @@
         <v>20</v>
       </c>
       <c r="R16" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S16">
         <v>39</v>
@@ -3130,7 +3130,7 @@
         <v>18</v>
       </c>
       <c r="W16" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X16">
         <v>58</v>
@@ -3145,7 +3145,7 @@
         <v>10</v>
       </c>
       <c r="AB16" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC16">
         <v>52</v>
@@ -3160,7 +3160,7 @@
         <v>15</v>
       </c>
       <c r="AG16" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH16">
         <v>58</v>
@@ -3175,7 +3175,7 @@
         <v>10</v>
       </c>
       <c r="AL16" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM16">
         <v>58</v>
@@ -3212,16 +3212,16 @@
         <v>112248</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="E17" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="F17" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="G17" s="3">
         <v>38853</v>
@@ -3231,19 +3231,19 @@
         <v>ABC-112248</v>
       </c>
       <c r="I17" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J17" s="1">
         <v>43952</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L17">
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N17">
         <v>32</v>
@@ -3258,7 +3258,7 @@
         <v>23</v>
       </c>
       <c r="R17" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S17">
         <v>52</v>
@@ -3273,7 +3273,7 @@
         <v>15</v>
       </c>
       <c r="W17" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X17">
         <v>42</v>
@@ -3288,7 +3288,7 @@
         <v>22</v>
       </c>
       <c r="AB17" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC17">
         <v>73</v>
@@ -3303,7 +3303,7 @@
         <v>23</v>
       </c>
       <c r="AG17" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH17">
         <v>42</v>
@@ -3318,7 +3318,7 @@
         <v>22</v>
       </c>
       <c r="AL17" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM17">
         <v>73</v>
@@ -3355,16 +3355,16 @@
         <v>112249</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="D18" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="E18" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="F18" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G18" s="3">
         <v>38854</v>
@@ -3374,19 +3374,19 @@
         <v>ABC-112249</v>
       </c>
       <c r="I18" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J18" s="1">
         <v>43952</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L18">
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N18">
         <v>54</v>
@@ -3401,7 +3401,7 @@
         <v>22</v>
       </c>
       <c r="R18" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S18">
         <v>73</v>
@@ -3416,7 +3416,7 @@
         <v>23</v>
       </c>
       <c r="W18" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X18">
         <v>32</v>
@@ -3431,7 +3431,7 @@
         <v>22</v>
       </c>
       <c r="AB18" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC18">
         <v>32</v>
@@ -3446,7 +3446,7 @@
         <v>22</v>
       </c>
       <c r="AG18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH18">
         <v>52</v>
@@ -3461,7 +3461,7 @@
         <v>15</v>
       </c>
       <c r="AL18" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM18">
         <v>32</v>
@@ -3498,16 +3498,16 @@
         <v>112250</v>
       </c>
       <c r="C19" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="D19" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="E19" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F19" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="G19" s="3">
         <v>38855</v>
@@ -3517,19 +3517,19 @@
         <v>ABC-112250</v>
       </c>
       <c r="I19" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J19" s="1">
         <v>43952</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L19">
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N19">
         <v>16</v>
@@ -3544,7 +3544,7 @@
         <v>19</v>
       </c>
       <c r="R19" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S19">
         <v>58</v>
@@ -3559,7 +3559,7 @@
         <v>10</v>
       </c>
       <c r="W19" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X19">
         <v>35</v>
@@ -3574,7 +3574,7 @@
         <v>20</v>
       </c>
       <c r="AB19" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC19">
         <v>35</v>
@@ -3589,7 +3589,7 @@
         <v>20</v>
       </c>
       <c r="AG19" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH19">
         <v>58</v>
@@ -3604,7 +3604,7 @@
         <v>10</v>
       </c>
       <c r="AL19" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM19">
         <v>35</v>
@@ -3641,16 +3641,16 @@
         <v>112251</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="D20" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="E20" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="F20" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="G20" s="3">
         <v>38856</v>
@@ -3660,19 +3660,19 @@
         <v>ABC-112251</v>
       </c>
       <c r="I20" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J20" s="1">
         <v>43952</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L20">
         <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N20">
         <v>68</v>
@@ -3687,7 +3687,7 @@
         <v>24</v>
       </c>
       <c r="R20" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S20">
         <v>42</v>
@@ -3702,7 +3702,7 @@
         <v>22</v>
       </c>
       <c r="W20" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X20">
         <v>52</v>
@@ -3717,7 +3717,7 @@
         <v>15</v>
       </c>
       <c r="AB20" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC20">
         <v>52</v>
@@ -3732,7 +3732,7 @@
         <v>15</v>
       </c>
       <c r="AG20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH20">
         <v>73</v>
@@ -3747,7 +3747,7 @@
         <v>23</v>
       </c>
       <c r="AL20" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM20">
         <v>58</v>
@@ -3784,16 +3784,16 @@
         <v>112252</v>
       </c>
       <c r="C21" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="D21" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E21" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F21" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="G21" s="3">
         <v>38857</v>
@@ -3803,19 +3803,19 @@
         <v>ABC-112252</v>
       </c>
       <c r="I21" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J21" s="1">
         <v>43952</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L21">
         <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N21">
         <v>39</v>
@@ -3830,7 +3830,7 @@
         <v>18</v>
       </c>
       <c r="R21" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S21">
         <v>32</v>
@@ -3845,7 +3845,7 @@
         <v>22</v>
       </c>
       <c r="W21" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X21">
         <v>73</v>
@@ -3860,7 +3860,7 @@
         <v>23</v>
       </c>
       <c r="AB21" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC21">
         <v>58</v>
@@ -3875,7 +3875,7 @@
         <v>10</v>
       </c>
       <c r="AG21" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH21">
         <v>32</v>
@@ -3890,7 +3890,7 @@
         <v>22</v>
       </c>
       <c r="AL21" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM21">
         <v>73</v>
@@ -3927,16 +3927,16 @@
         <v>112253</v>
       </c>
       <c r="C22" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D22" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="E22" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="F22" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="G22" s="3">
         <v>38858</v>
@@ -3946,19 +3946,19 @@
         <v>ABC-112253</v>
       </c>
       <c r="I22" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J22" s="1">
         <v>43952</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L22">
         <v>1</v>
       </c>
       <c r="M22" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N22">
         <v>52</v>
@@ -3973,7 +3973,7 @@
         <v>15</v>
       </c>
       <c r="R22" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S22">
         <v>35</v>
@@ -3988,7 +3988,7 @@
         <v>20</v>
       </c>
       <c r="W22" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X22">
         <v>32</v>
@@ -4003,7 +4003,7 @@
         <v>22</v>
       </c>
       <c r="AB22" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC22">
         <v>42</v>
@@ -4018,7 +4018,7 @@
         <v>22</v>
       </c>
       <c r="AG22" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH22">
         <v>35</v>
@@ -4033,7 +4033,7 @@
         <v>20</v>
       </c>
       <c r="AL22" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM22">
         <v>32</v>
@@ -4070,16 +4070,16 @@
         <v>112254</v>
       </c>
       <c r="C23" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D23" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="E23" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="F23" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="G23" s="3">
         <v>38859</v>
@@ -4089,19 +4089,19 @@
         <v>ABC-112254</v>
       </c>
       <c r="I23" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J23" s="1">
         <v>43952</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L23">
         <v>1</v>
       </c>
       <c r="M23" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N23">
         <v>73</v>
@@ -4116,7 +4116,7 @@
         <v>23</v>
       </c>
       <c r="R23" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S23">
         <v>52</v>
@@ -4131,7 +4131,7 @@
         <v>15</v>
       </c>
       <c r="W23" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X23">
         <v>35</v>
@@ -4146,7 +4146,7 @@
         <v>20</v>
       </c>
       <c r="AB23" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC23">
         <v>52</v>
@@ -4161,7 +4161,7 @@
         <v>15</v>
       </c>
       <c r="AG23" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH23">
         <v>52</v>
@@ -4176,7 +4176,7 @@
         <v>15</v>
       </c>
       <c r="AL23" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM23">
         <v>35</v>
@@ -4213,16 +4213,16 @@
         <v>112255</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="D24" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="E24" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="F24" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="G24" s="3">
         <v>38860</v>
@@ -4232,19 +4232,19 @@
         <v>ABC-112255</v>
       </c>
       <c r="I24" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J24" s="1">
         <v>43952</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L24">
         <v>1</v>
       </c>
       <c r="M24" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N24">
         <v>58</v>
@@ -4259,7 +4259,7 @@
         <v>10</v>
       </c>
       <c r="R24" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S24">
         <v>73</v>
@@ -4274,7 +4274,7 @@
         <v>23</v>
       </c>
       <c r="W24" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X24">
         <v>52</v>
@@ -4289,7 +4289,7 @@
         <v>15</v>
       </c>
       <c r="AB24" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC24">
         <v>58</v>
@@ -4304,7 +4304,7 @@
         <v>10</v>
       </c>
       <c r="AG24" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH24">
         <v>58</v>
@@ -4319,7 +4319,7 @@
         <v>10</v>
       </c>
       <c r="AL24" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM24">
         <v>58</v>
@@ -4356,16 +4356,16 @@
         <v>112256</v>
       </c>
       <c r="C25" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D25" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E25" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="F25" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="G25" s="3">
         <v>38861</v>
@@ -4375,19 +4375,19 @@
         <v>ABC-112256</v>
       </c>
       <c r="I25" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J25" s="1">
         <v>43952</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L25">
         <v>1</v>
       </c>
       <c r="M25" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N25">
         <v>42</v>
@@ -4402,7 +4402,7 @@
         <v>22</v>
       </c>
       <c r="R25" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S25">
         <v>58</v>
@@ -4417,7 +4417,7 @@
         <v>10</v>
       </c>
       <c r="W25" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X25">
         <v>58</v>
@@ -4432,7 +4432,7 @@
         <v>10</v>
       </c>
       <c r="AB25" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC25">
         <v>73</v>
@@ -4447,7 +4447,7 @@
         <v>23</v>
       </c>
       <c r="AG25" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH25">
         <v>58</v>
@@ -4462,7 +4462,7 @@
         <v>10</v>
       </c>
       <c r="AL25" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM25">
         <v>73</v>
@@ -4499,16 +4499,16 @@
         <v>112257</v>
       </c>
       <c r="C26" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D26" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="E26" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="F26" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="G26" s="3">
         <v>38862</v>
@@ -4518,19 +4518,19 @@
         <v>ABC-112257</v>
       </c>
       <c r="I26" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J26" s="1">
         <v>43952</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="L26">
         <v>1</v>
       </c>
       <c r="M26" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N26">
         <v>32</v>
@@ -4545,7 +4545,7 @@
         <v>22</v>
       </c>
       <c r="R26" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="S26">
         <v>42</v>
@@ -4560,7 +4560,7 @@
         <v>22</v>
       </c>
       <c r="W26" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="X26">
         <v>42</v>
@@ -4575,7 +4575,7 @@
         <v>22</v>
       </c>
       <c r="AB26" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="AC26">
         <v>32</v>
@@ -4590,7 +4590,7 @@
         <v>22</v>
       </c>
       <c r="AG26" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="AH26">
         <v>73</v>
@@ -4605,7 +4605,7 @@
         <v>23</v>
       </c>
       <c r="AL26" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AM26">
         <v>32</v>

</xml_diff>